<commit_message>
log fix and upload file fixes
</commit_message>
<xml_diff>
--- a/sample_templates/Add_Users.xlsx
+++ b/sample_templates/Add_Users.xlsx
@@ -7,7 +7,7 @@
     <workbookView windowWidth="19200" windowHeight="6800"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Add Users" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,33 +27,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
-  <si>
-    <t>UserName</t>
-  </si>
-  <si>
-    <t>ManagerIDs</t>
-  </si>
-  <si>
-    <t>ContactNumber</t>
-  </si>
-  <si>
-    <t>RoleId</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
+  <si>
+    <t>Company ID</t>
+  </si>
+  <si>
+    <t>User Name</t>
+  </si>
+  <si>
+    <t>Manager IDs</t>
+  </si>
+  <si>
+    <t>Contact</t>
+  </si>
+  <si>
+    <t>User Role ID</t>
   </si>
   <si>
     <t>Email</t>
   </si>
   <si>
-    <t>CountryCode</t>
-  </si>
-  <si>
-    <t>countryIsoCode</t>
-  </si>
-  <si>
-    <t>LocationName</t>
-  </si>
-  <si>
-    <t>TimeZone</t>
+    <t>Country Code (ISD)</t>
+  </si>
+  <si>
+    <t>Country ISO Code</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Time Zone</t>
   </si>
   <si>
     <t>Language</t>
@@ -62,31 +65,67 @@
     <t>Currency</t>
   </si>
   <si>
-    <t>AreaUnits</t>
-  </si>
-  <si>
-    <t>Locale</t>
-  </si>
-  <si>
-    <t>John Doe</t>
-  </si>
-  <si>
-    <t>123</t>
-  </si>
-  <si>
-    <t>9876543210</t>
-  </si>
-  <si>
-    <t>101</t>
-  </si>
-  <si>
-    <t>john@example.com</t>
+    <t>Area Units</t>
+  </si>
+  <si>
+    <t>Locale Settings</t>
+  </si>
+  <si>
+    <t>Plan Type Preference</t>
+  </si>
+  <si>
+    <t>Crop Preference</t>
+  </si>
+  <si>
+    <t>Project Preference</t>
+  </si>
+  <si>
+    <t>Forms</t>
+  </si>
+  <si>
+    <t>Location Preference</t>
+  </si>
+  <si>
+    <t>Farmer Tags</t>
+  </si>
+  <si>
+    <t>Asset Tags</t>
+  </si>
+  <si>
+    <t>Plot Tags</t>
+  </si>
+  <si>
+    <t>Precipitation Unit</t>
+  </si>
+  <si>
+    <t>Temperature Unit</t>
+  </si>
+  <si>
+    <t>Weight Unit</t>
+  </si>
+  <si>
+    <t>Geo ID</t>
+  </si>
+  <si>
+    <t>test automation 01</t>
+  </si>
+  <si>
+    <t>2978903, 1289651</t>
+  </si>
+  <si>
+    <t>7382218237</t>
+  </si>
+  <si>
+    <t>test@example.com</t>
   </si>
   <si>
     <t>IN</t>
   </si>
   <si>
-    <t>Bangalore</t>
+    <t>Accepts:
+City Names: Bangalore | Nellore
+Coordinates: 12.663, 44.772 | 66.77, 88.22
+Mixed: Bangalore | 12.9716, 77.5946 | Nellore</t>
   </si>
   <si>
     <t>IST</t>
@@ -98,10 +137,40 @@
     <t>INR</t>
   </si>
   <si>
-    <t>HECTARE</t>
+    <t>ACRE</t>
   </si>
   <si>
     <t>en-IN</t>
+  </si>
+  <si>
+    <t>3880752, 3876003</t>
+  </si>
+  <si>
+    <t>1841751, 3438752</t>
+  </si>
+  <si>
+    <t>3182652</t>
+  </si>
+  <si>
+    <t>3745552, 3691952</t>
+  </si>
+  <si>
+    <t>3808252, 3770307</t>
+  </si>
+  <si>
+    <t>3811552</t>
+  </si>
+  <si>
+    <t>3811553</t>
+  </si>
+  <si>
+    <t>Inches</t>
+  </si>
+  <si>
+    <t>Celsius</t>
+  </si>
+  <si>
+    <t>Tonne</t>
   </si>
 </sst>
 </file>
@@ -281,7 +350,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -290,6 +359,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -475,27 +550,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -620,7 +680,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -632,122 +692,128 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1095,95 +1161,194 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="1"/>
   <cols>
-    <col min="2" max="2" width="11.9090909090909" customWidth="1"/>
-    <col min="3" max="3" width="15.5454545454545" customWidth="1"/>
-    <col min="6" max="6" width="12.9090909090909" customWidth="1"/>
-    <col min="7" max="8" width="14" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="23" customWidth="1"/>
+    <col min="8" max="8" width="21" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
+    <col min="11" max="12" width="13" customWidth="1"/>
+    <col min="13" max="13" width="15" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
+    <col min="15" max="15" width="25" customWidth="1"/>
+    <col min="16" max="16" width="20" customWidth="1"/>
+    <col min="17" max="17" width="23" customWidth="1"/>
+    <col min="18" max="18" width="10" customWidth="1"/>
+    <col min="19" max="19" width="24" customWidth="1"/>
+    <col min="20" max="20" width="16" customWidth="1"/>
+    <col min="21" max="21" width="15" customWidth="1"/>
+    <col min="22" max="22" width="14" customWidth="1"/>
+    <col min="23" max="23" width="23" customWidth="1"/>
+    <col min="24" max="24" width="21" customWidth="1"/>
+    <col min="25" max="25" width="16" customWidth="1"/>
+    <col min="26" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:26">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:13">
-      <c r="A2" t="s">
-        <v>13</v>
+    <row r="2" ht="174" spans="1:26">
+      <c r="A2">
+        <v>1251</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2">
+        <v>28</v>
+      </c>
+      <c r="E2">
+        <v>1351</v>
+      </c>
+      <c r="F2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2">
         <v>91</v>
       </c>
-      <c r="G2" t="s">
-        <v>18</v>
-      </c>
       <c r="H2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" t="s">
-        <v>20</v>
+        <v>30</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="J2" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="K2" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="L2" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="M2" t="s">
-        <v>24</v>
+        <v>35</v>
+      </c>
+      <c r="N2" t="s">
+        <v>36</v>
+      </c>
+      <c r="O2" t="s">
+        <v>37</v>
+      </c>
+      <c r="P2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>39</v>
+      </c>
+      <c r="R2" t="s">
+        <v>40</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="T2" t="s">
+        <v>41</v>
+      </c>
+      <c r="U2" t="s">
+        <v>42</v>
+      </c>
+      <c r="V2" t="s">
+        <v>43</v>
+      </c>
+      <c r="W2" t="s">
+        <v>44</v>
+      </c>
+      <c r="X2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>46</v>
+      </c>
+      <c r="Z2">
+        <v>656497</v>
       </c>
     </row>
   </sheetData>

</xml_diff>